<commit_message>
Grafiken mit Datenbeschriftung: Werte auf Balken, Werte+Prozent+Kategorie auf Kuchen
</commit_message>
<xml_diff>
--- a/docs/latest_report.xlsx
+++ b/docs/latest_report.xlsx
@@ -223,6 +223,10 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -335,6 +339,11 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="1"/>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>
     </plotArea>
@@ -703,7 +712,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46103.54655185567</v>
+        <v>46103.5502430104</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
3 neue Artikel (Der Standard, fixed-income, Finews/Savchenko)
</commit_message>
<xml_diff>
--- a/docs/latest_report.xlsx
+++ b/docs/latest_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -177,14 +177,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -208,7 +208,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -240,8 +240,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -267,8 +267,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -294,14 +294,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -324,7 +324,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -357,12 +357,12 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="3600000"/>
@@ -372,9 +372,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -384,7 +384,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="3600000"/>
@@ -394,9 +394,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -712,7 +712,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46104.36153620944</v>
+        <v>46104.53151494826</v>
       </c>
     </row>
     <row r="8">
@@ -754,21 +754,21 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>46100</v>
+        <v>46102</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Moneycab</t>
+          <t>Der Standard</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Nicht nur Öl: Wo der Iran-Konflikt Emerging Markets wirklich trifft</t>
+          <t>Pakistan spart Milliarden an fossilen Importen: Wie hat es das gemacht?</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -777,31 +777,31 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>https://www.moneycab.com/finanz/nicht-nur-oel-wo-der-iran-konflikt-emerging-markets-wirklich-trifft/</t>
+          <t>https://www.derstandard.de/story/3000000313347/pakistan-spart-milliarden-an-fossilen-importen-wie-hat-es-das-gemacht</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>46100</v>
+        <v>46102</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Institutional Money</t>
+          <t>Finews</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
+          <t>Tokenisierung: Louzia Savchenko ueber Innovation und MK Global Kapital</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -814,27 +814,27 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.institutional-money.com/news/maerkte/headline/was-der-iran-schock-fuer-emerging-markets-veraendert-249420</t>
+          <t>https://www.finews.ch/news/finanzplatz/71578-finews-first-tokenisierung-louzia-savchenko-finanzplatz-schweiz-innovation-mk-global-kapital</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>46098</v>
+        <v>46100</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>finanznachrichten.de</t>
+          <t>Moneycab</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Private Credit ist nicht gleich Private Credit: Wo die Risiken wirklich liegen</t>
+          <t>Nicht nur Öl: Wo der Iran-Konflikt Emerging Markets wirklich trifft</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -847,22 +847,22 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.finanznachrichten.de/nachrichten-2026-03/67998176-private-credit-ist-nicht-gleich-private-credit-wo-die-risiken-wirklich-liegen-144.htm</t>
+          <t>https://www.moneycab.com/finanz/nicht-nur-oel-wo-der-iran-konflikt-emerging-markets-wirklich-trifft/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>46098</v>
+        <v>46100</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>cash-online.de</t>
+          <t>Institutional Money</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Gastkommentar: Der blinde Fleck der Private-Credit-Debatte</t>
+          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -876,26 +876,26 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://www.cash-online.de/a/gastkommentar-der-blinde-fleck-der-private-credit-debatte-713724/</t>
+          <t>https://www.institutional-money.com/news/maerkte/headline/was-der-iran-schock-fuer-emerging-markets-veraendert-249420</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>FONDS exklusiv</t>
+          <t>fixed-income.org</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Private Credit-Debatte entfacht</t>
+          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -913,22 +913,22 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
+          <t>https://www.fixed-income.org/investment/was-der-iran-schock-fuer-emerging-markets-veraendert.html</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Anlageklasse</t>
+          <t>Private Credit ist nicht gleich Private Credit: Wo die Risiken wirklich liegen</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Print &amp; Online</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
@@ -946,27 +946,27 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-03/67998176-private-credit-ist-nicht-gleich-private-credit-wo-die-risiken-wirklich-liegen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>46091</v>
+        <v>46098</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Swiss Finance AI</t>
+          <t>cash-online.de</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Warum tokenisierte Anleihen mehr sind als ein Trend</t>
+          <t>Gastkommentar: Der blinde Fleck der Private-Credit-Debatte</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -979,22 +979,22 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://www.swissfinanceai.ch/blog/swiss-finance/warum-tokenisierte-anleihen-mehr-sind-als-ein-trend</t>
+          <t>https://www.cash-online.de/a/gastkommentar-der-blinde-fleck-der-private-credit-debatte-713724/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>46085</v>
+        <v>46097</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>markteinblicke.de</t>
+          <t>FONDS exklusiv</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
+          <t>Private Credit-Debatte entfacht</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1008,26 +1008,26 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
+          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>46085</v>
+        <v>46097</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>gruenderkueche.de</t>
+          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
+          <t>Mikrofinanz als Anlageklasse</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print &amp; Online</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
@@ -1045,27 +1045,27 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
+          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>46083</v>
+        <v>46091</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>altii.de</t>
+          <t>Swiss Finance AI</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
+          <t>Warum tokenisierte Anleihen mehr sind als ein Trend</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1074,26 +1074,26 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
+          <t>https://www.swissfinanceai.ch/blog/swiss-finance/warum-tokenisierte-anleihen-mehr-sind-als-ein-trend</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>46077</v>
+        <v>46085</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>markteinblicke.de</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1107,26 +1107,26 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
+          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>46076</v>
+        <v>46085</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>exxecnews.org</t>
+          <t>gruenderkueche.de</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1144,22 +1144,22 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
+          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>46071</v>
+        <v>46083</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>altii.de</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
+          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1173,31 +1173,31 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
+          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>46069</v>
+        <v>46077</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Börsen-Kurier</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
+          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1208,20 +1208,24 @@
       <c r="F22" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>46067</v>
+        <v>46076</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>finanznachrichten.de</t>
+          <t>exxecnews.org</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1239,22 +1243,22 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
+          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>46067</v>
+        <v>46071</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1272,27 +1276,27 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
+          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>46067</v>
+        <v>46069</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>geldmeisterin.com</t>
+          <t>Börsen-Kurier</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
+          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1303,29 +1307,25 @@
       <c r="F25" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
-        </is>
-      </c>
+      <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>46057</v>
+        <v>46067</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1338,27 +1338,27 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>46055</v>
+        <v>46067</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>bondguide.de</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1371,22 +1371,22 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
+          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>46049</v>
+        <v>46067</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>geldmeisterin.com</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1396,31 +1396,35 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>46044</v>
+        <v>46057</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Frankfurter Allgemeine Zeitung</t>
+          <t>investrends.ch</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
+          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1429,31 +1433,31 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
+          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>46038</v>
+        <v>46055</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>E-fundresearch</t>
+          <t>Payoff</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
+          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1466,55 +1470,51 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
+          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>46035</v>
+        <v>46049</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>Markt Einblicke</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>46029</v>
+        <v>46044</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>Frankfurter Allgemeine Zeitung</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1528,31 +1528,31 @@
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
+          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>46028</v>
+        <v>46038</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>portfolio institutionell</t>
+          <t>E-fundresearch</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Große Wirkung mit kleinen Krediten</t>
+          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1561,26 +1561,26 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
+          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>46000</v>
+        <v>46035</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>Finews</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1594,31 +1594,31 @@
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
+          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>45999</v>
+        <v>46029</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Moneycab</t>
+          <t>Markt Einblicke</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -1631,22 +1631,22 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
+          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>45997</v>
+        <v>46028</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>portfolio institutionell</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+          <t>Große Wirkung mit kleinen Krediten</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1660,26 +1660,26 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+          <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>45985</v>
+        <v>46000</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>investrends.ch</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1693,26 +1693,26 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>45973</v>
+        <v>45999</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>Moneycab</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1730,38 +1730,137 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
+        <v>45997</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>bondguide.de</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Finews</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>45973</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>investrends.ch</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
         <v>45848</v>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Handelszeitung</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Zwischen ESG-Müdigkeit und Wirkungsanspruch</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="n">
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>https://www.handelszeitung.ch/specials/nachhaltiges-investieren-2024/zwischen-esg-mudigkeit-und-wirkungsanspruch-841576</t>
         </is>
@@ -1781,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1802,7 +1901,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Source: Sheet '2026 Clippings' (A9:G39)</t>
+          <t>Source: Sheet '2026 Clippings' (A9:G42)</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1919,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -1840,7 +1939,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>46100</v>
+        <v>46102</v>
       </c>
     </row>
     <row r="8">
@@ -1850,7 +1949,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -1860,7 +1959,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1909,10 +2008,10 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.2580645161290323</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
@@ -1930,10 +2029,10 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.7419354838709677</v>
+        <v>0.7058823529411765</v>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
@@ -1981,7 +2080,7 @@
         </is>
       </c>
       <c r="F17" s="8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
@@ -2031,14 +2130,14 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>0.3225806451612903</v>
+        <v>0.02941176470588235</v>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
@@ -2046,23 +2145,23 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>0.9354838709677419</v>
+        <v>0.9411764705882353</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
@@ -2073,20 +2172,20 @@
         <v>1</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>0.03225806451612903</v>
+        <v>0.02941176470588235</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0.06451612903225806</v>
+        <v>0.5882352941176471</v>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
@@ -2097,7 +2196,20 @@
         <v>1</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>0.03225806451612903</v>
+        <v>0.02941176470588235</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>DACH</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>0.05882352941176471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Google Search API + 3 neue Artikel (FAZ, DAS INVESTMENT, FONDS exklusiv AT)
</commit_message>
<xml_diff>
--- a/docs/latest_report.xlsx
+++ b/docs/latest_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -177,14 +177,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -208,7 +208,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -240,8 +240,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -267,8 +267,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -294,14 +294,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -324,7 +324,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -357,7 +357,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -372,9 +372,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -394,9 +394,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -712,7 +712,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46106.3394595858</v>
+        <v>46106.38656813572</v>
       </c>
     </row>
     <row r="8">
@@ -754,21 +754,21 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Der Standard</t>
+          <t>Frankfurter Allgemeine Zeitung</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Pakistan spart Milliarden an fossilen Importen: Wie hat es das gemacht?</t>
+          <t>Sorgen um Privatkredite: Finanzkrise oder silberne Aera?</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -781,27 +781,27 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>https://www.derstandard.de/story/3000000313347/pakistan-spart-milliarden-an-fossilen-importen-wie-hat-es-das-gemacht</t>
+          <t>https://www.faz.net/pro/meine-finanzen/zinsen/sorgen-um-privatkredite-finanzkrise-oder-silberne-aera-110376123.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>DAS INVESTMENT</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Tokenisierung: Louzia Savchenko ueber Innovation und MK Global Kapital</t>
+          <t>Private Credit unter Druck: Wenn das Geld nicht mehr herauskommt</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -814,27 +814,27 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.finews.ch/news/finanzplatz/71578-finews-first-tokenisierung-louzia-savchenko-finanzplatz-schweiz-innovation-mk-global-kapital</t>
+          <t>https://www.dasinvestment.com/private-credit-unter-druck-wenn-das-geld-nicht-mehr-herauskommt/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>46100</v>
+        <v>46105</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Moneycab</t>
+          <t>FONDS exklusiv Oesterreich</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Nicht nur Öl: Wo der Iran-Konflikt Emerging Markets wirklich trifft</t>
+          <t>Private Credit-Debatte entfacht</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -847,27 +847,27 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.moneycab.com/finanz/nicht-nur-oel-wo-der-iran-konflikt-emerging-markets-wirklich-trifft/</t>
+          <t>https://www.fondsexklusiv.at/private-credit-debatte-entfacht/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>46100</v>
+        <v>46102</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Institutional Money</t>
+          <t>Der Standard</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
+          <t>Pakistan spart Milliarden an fossilen Importen: Wie hat es das gemacht?</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -880,27 +880,27 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://www.institutional-money.com/news/maerkte/headline/was-der-iran-schock-fuer-emerging-markets-veraendert-249420</t>
+          <t>https://www.derstandard.de/story/3000000313347/pakistan-spart-milliarden-an-fossilen-importen-wie-hat-es-das-gemacht</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>46100</v>
+        <v>46102</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>fixed-income.org</t>
+          <t>Finews</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
+          <t>Tokenisierung: Louzia Savchenko ueber Innovation und MK Global Kapital</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -909,31 +909,31 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.fixed-income.org/investment/was-der-iran-schock-fuer-emerging-markets-veraendert.html</t>
+          <t>https://www.finews.ch/news/finanzplatz/71578-finews-first-tokenisierung-louzia-savchenko-finanzplatz-schweiz-innovation-mk-global-kapital</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>46098</v>
+        <v>46100</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>finanznachrichten.de</t>
+          <t>Moneycab</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Private Credit ist nicht gleich Private Credit: Wo die Risiken wirklich liegen</t>
+          <t>Nicht nur Öl: Wo der Iran-Konflikt Emerging Markets wirklich trifft</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.finanznachrichten.de/nachrichten-2026-03/67998176-private-credit-ist-nicht-gleich-private-credit-wo-die-risiken-wirklich-liegen-144.htm</t>
+          <t>https://www.moneycab.com/finanz/nicht-nur-oel-wo-der-iran-konflikt-emerging-markets-wirklich-trifft/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>46098</v>
+        <v>46100</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>cash-online.de</t>
+          <t>Institutional Money</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Gastkommentar: Der blinde Fleck der Private-Credit-Debatte</t>
+          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -975,26 +975,26 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://www.cash-online.de/a/gastkommentar-der-blinde-fleck-der-private-credit-debatte-713724/</t>
+          <t>https://www.institutional-money.com/news/maerkte/headline/was-der-iran-schock-fuer-emerging-markets-veraendert-249420</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>FONDS exklusiv</t>
+          <t>fixed-income.org</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Private Credit-Debatte entfacht</t>
+          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1012,22 +1012,22 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
+          <t>https://www.fixed-income.org/investment/was-der-iran-schock-fuer-emerging-markets-veraendert.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Anlageklasse</t>
+          <t>Private Credit ist nicht gleich Private Credit: Wo die Risiken wirklich liegen</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Print &amp; Online</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
@@ -1045,27 +1045,27 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-03/67998176-private-credit-ist-nicht-gleich-private-credit-wo-die-risiken-wirklich-liegen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>46091</v>
+        <v>46098</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Swiss Finance AI</t>
+          <t>cash-online.de</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Warum tokenisierte Anleihen mehr sind als ein Trend</t>
+          <t>Gastkommentar: Der blinde Fleck der Private-Credit-Debatte</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1078,22 +1078,22 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>https://www.swissfinanceai.ch/blog/swiss-finance/warum-tokenisierte-anleihen-mehr-sind-als-ein-trend</t>
+          <t>https://www.cash-online.de/a/gastkommentar-der-blinde-fleck-der-private-credit-debatte-713724/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>46085</v>
+        <v>46097</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>markteinblicke.de</t>
+          <t>FONDS exklusiv</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
+          <t>Private Credit-Debatte entfacht</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1107,26 +1107,26 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
+          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>46085</v>
+        <v>46097</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>gruenderkueche.de</t>
+          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
+          <t>Mikrofinanz als Anlageklasse</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print &amp; Online</t>
         </is>
       </c>
       <c r="F20" s="4" t="n">
@@ -1144,27 +1144,27 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
+          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>46083</v>
+        <v>46091</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>altii.de</t>
+          <t>Swiss Finance AI</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
+          <t>Warum tokenisierte Anleihen mehr sind als ein Trend</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1173,26 +1173,26 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
+          <t>https://www.swissfinanceai.ch/blog/swiss-finance/warum-tokenisierte-anleihen-mehr-sind-als-ein-trend</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>46077</v>
+        <v>46085</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>markteinblicke.de</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1206,26 +1206,26 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
+          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>46076</v>
+        <v>46085</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>exxecnews.org</t>
+          <t>gruenderkueche.de</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1243,22 +1243,22 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
+          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>46071</v>
+        <v>46083</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>altii.de</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
+          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1272,31 +1272,31 @@
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
+          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>46069</v>
+        <v>46077</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Börsen-Kurier</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
+          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1307,20 +1307,24 @@
       <c r="F25" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>46067</v>
+        <v>46076</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>finanznachrichten.de</t>
+          <t>exxecnews.org</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1338,22 +1342,22 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
+          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>46067</v>
+        <v>46071</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1371,27 +1375,27 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
+          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>46067</v>
+        <v>46069</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>geldmeisterin.com</t>
+          <t>Börsen-Kurier</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
+          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1402,29 +1406,25 @@
       <c r="F28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
-        </is>
-      </c>
+      <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>46057</v>
+        <v>46067</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1437,27 +1437,27 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>46055</v>
+        <v>46067</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>bondguide.de</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1470,22 +1470,22 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
+          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>46049</v>
+        <v>46067</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>geldmeisterin.com</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1495,31 +1495,35 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>46044</v>
+        <v>46057</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Frankfurter Allgemeine Zeitung</t>
+          <t>investrends.ch</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
+          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1528,31 +1532,31 @@
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
+          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>46038</v>
+        <v>46055</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>E-fundresearch</t>
+          <t>Payoff</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
+          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1565,55 +1569,51 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
+          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>46035</v>
+        <v>46049</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>Markt Einblicke</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>46029</v>
+        <v>46044</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>Frankfurter Allgemeine Zeitung</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1627,31 +1627,31 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
+          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>46028</v>
+        <v>46038</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>portfolio institutionell</t>
+          <t>E-fundresearch</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Große Wirkung mit kleinen Krediten</t>
+          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -1660,26 +1660,26 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
+          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>46000</v>
+        <v>46035</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>Finews</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
+          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>45999</v>
+        <v>46029</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Moneycab</t>
+          <t>Markt Einblicke</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -1730,22 +1730,22 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
+          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>45997</v>
+        <v>46028</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>portfolio institutionell</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+          <t>Große Wirkung mit kleinen Krediten</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1759,26 +1759,26 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+          <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>45985</v>
+        <v>46000</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>investrends.ch</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1792,26 +1792,26 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
-        <v>45973</v>
+        <v>45999</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>Moneycab</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1829,38 +1829,137 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
+        <v>45997</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>bondguide.de</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Finews</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>45973</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>investrends.ch</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
         <v>45848</v>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>Handelszeitung</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Zwischen ESG-Müdigkeit und Wirkungsanspruch</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="n">
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>https://www.handelszeitung.ch/specials/nachhaltiges-investieren-2024/zwischen-esg-mudigkeit-und-wirkungsanspruch-841576</t>
         </is>
@@ -1901,7 +2000,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Source: Sheet '2026 Clippings' (A9:G42)</t>
+          <t>Source: Sheet '2026 Clippings' (A9:G45)</t>
         </is>
       </c>
     </row>
@@ -1919,7 +2018,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -1939,7 +2038,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>46102</v>
+        <v>46105</v>
       </c>
     </row>
     <row r="8">
@@ -1949,7 +2048,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -2008,10 +2107,10 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.3243243243243243</v>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
@@ -2029,10 +2128,10 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
@@ -2080,7 +2179,7 @@
         </is>
       </c>
       <c r="F17" s="8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22">
@@ -2134,10 +2233,10 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.05405405405405406</v>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
@@ -2145,10 +2244,10 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9459459459459459</v>
       </c>
     </row>
     <row r="25">
@@ -2161,7 +2260,7 @@
         <v>11</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.2972972972972973</v>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
@@ -2172,7 +2271,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="26">
@@ -2182,10 +2281,10 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.5945945945945946</v>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
@@ -2196,7 +2295,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="27">
@@ -2209,7 +2308,7 @@
         <v>2</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bugfixes: fehlende IDs, ungenutzter Import, Datenintegritaet
</commit_message>
<xml_diff>
--- a/docs/latest_report.xlsx
+++ b/docs/latest_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -177,14 +177,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -208,7 +208,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -240,8 +240,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -267,8 +267,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -294,14 +294,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -324,7 +324,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -357,7 +357,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -372,9 +372,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -394,9 +394,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -712,7 +712,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46111.44689778658</v>
+        <v>46111.63234792282</v>
       </c>
     </row>
     <row r="8">

</xml_diff>